<commit_message>
app now is MAN-friendly
</commit_message>
<xml_diff>
--- a/data/clients.xlsx
+++ b/data/clients.xlsx
@@ -442,62 +442,62 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>Создан</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>Обновлен</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>client_name</t>
+          <t>Клиент</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>folder</t>
+          <t>Папка клиента</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>files_count</t>
+          <t>Файлов</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>last_file</t>
+          <t>Последний файл</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>full_name</t>
+          <t>ФИО</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>passport</t>
+          <t>Паспорт</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>inn</t>
+          <t>ИНН</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>Дата</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>last_template</t>
+          <t>Шаблон</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>last_document</t>
+          <t>Готовый документ</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added an excel table for clients
</commit_message>
<xml_diff>
--- a/data/clients.xlsx
+++ b/data/clients.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -501,6 +501,36 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-09-12 02:14:41</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-09-12 02:15:57</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>морф</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>data/clients/морф</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>data/clients/морф/морфморф.png</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>